<commit_message>
data(gis): publish GeoLibre analysis yilan-public-facility-hazard-exposure-2026-09
</commit_message>
<xml_diff>
--- a/GeoLibre-Web/analysis/yilan-public-facility-hazard-exposure-2026-09/result.xlsx
+++ b/GeoLibre-Web/analysis/yilan-public-facility-hazard-exposure-2026-09/result.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'分析結果'!$A$1:$V$112</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'統計摘要'!$A$1:$B$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'統計摘要'!$A$1:$B$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'分析參數'!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'資料來源'!$A$1:$K$11</definedName>
   </definedNames>
@@ -9464,7 +9464,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:15+00:00</t>
+          <t>2026-09-25T12:46:34+00:00</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -9544,7 +9544,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:15+00:00</t>
+          <t>2026-09-25T12:46:34+00:00</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -9624,7 +9624,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:15+00:00</t>
+          <t>2026-09-25T12:46:34+00:00</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -9704,7 +9704,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:15+00:00</t>
+          <t>2026-09-25T12:46:34+00:00</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -9784,7 +9784,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:15+00:00</t>
+          <t>2026-09-25T12:46:34+00:00</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -9864,7 +9864,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:15+00:00</t>
+          <t>2026-09-25T12:46:34+00:00</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -9944,7 +9944,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:15+00:00</t>
+          <t>2026-09-25T12:46:34+00:00</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -10008,7 +10008,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -10060,125 +10060,135 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>複合災害暴露設施數</t>
+          <t>敏感區內去重學校數</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>輸入設施類型：醫療機構</t>
+          <t>複合災害暴露設施數</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>42</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>輸入設施類型：政府機關</t>
+          <t>輸入設施類型：醫療機構</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>98</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>輸入設施類型：學校</t>
+          <t>輸入設施類型：政府機關</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>133</v>
+        <v>98</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>輸入設施類型：消防分隊</t>
+          <t>輸入設施類型：學校</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>18</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>設施類型：醫療機構</t>
+          <t>輸入設施類型：消防分隊</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>設施類型：政府機關</t>
+          <t>設施類型：醫療機構</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>設施類型：學校</t>
+          <t>設施類型：政府機關</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>設施類型：消防分隊</t>
+          <t>設施類型：學校</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>7</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>災害群組：土石流影響範圍</t>
+          <t>設施類型：消防分隊</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>28</v>
+        <v>7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>災害群組：地質敏感區</t>
+          <t>災害群組：土石流影響範圍</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>67</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>災害群組：地質敏感區</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>災害群組：近5年歷史淹水災點</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B17" t="n">
         <v>39</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B16"/>
+  <autoFilter ref="A1:B17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10286,7 +10296,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:27+00:00</t>
+          <t>2026-09-25T12:46:44+00:00</t>
         </is>
       </c>
     </row>
@@ -10399,7 +10409,7 @@
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:13+00:00</t>
+          <t>2026-09-25T12:46:33+00:00</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -10546,7 +10556,7 @@
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:14+00:00</t>
+          <t>2026-09-25T12:46:33+00:00</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -10595,7 +10605,7 @@
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:15+00:00</t>
+          <t>2026-09-25T12:46:34+00:00</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -10648,7 +10658,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:16+00:00</t>
+          <t>2026-09-25T12:46:35+00:00</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -10701,7 +10711,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:16+00:00</t>
+          <t>2026-09-25T12:46:35+00:00</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -10754,7 +10764,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:22+00:00</t>
+          <t>2026-09-25T12:46:41+00:00</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -10807,7 +10817,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:23+00:00</t>
+          <t>2026-09-25T12:46:41+00:00</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -10856,7 +10866,7 @@
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
-          <t>2026-09-25T12:42:26+00:00</t>
+          <t>2026-09-25T12:46:43+00:00</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">

</xml_diff>